<commit_message>
[Chore] 바뀐 엑셀 데이터에 따라 Gun Item Data 재파싱 (Sound Range 추가)
</commit_message>
<xml_diff>
--- a/Assets/06 Data/ExcelData/Gun_Item_Table.xlsx
+++ b/Assets/06 Data/ExcelData/Gun_Item_Table.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Genie\Desktop\duckov-clone\Assets\06 Data\ExcelData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\StudyUnity\Duckov\Assets\06 Data\ExcelData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{526B5CF3-02EA-4791-9198-AA3DBFDBEFB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78DE9398-3FC1-4E82-A6D3-ADB11DE44F07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3795" yWindow="3495" windowWidth="21600" windowHeight="11295" xr2:uid="{818AEAD1-047B-4735-8CBD-03FE823548AF}"/>
+    <workbookView xWindow="31920" yWindow="2490" windowWidth="18225" windowHeight="8595" xr2:uid="{818AEAD1-047B-4735-8CBD-03FE823548AF}"/>
   </bookViews>
   <sheets>
     <sheet name="무기" sheetId="1" r:id="rId1"/>
@@ -206,7 +206,7 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>soundRange</t>
+    <t>SoundRange</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>

</xml_diff>